<commit_message>
Update soccer trades 2026-08-02 06:02:30 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Superliga/trades.xlsx
+++ b/data/sxbet/ligas/Superliga/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V59"/>
+  <dimension ref="A1:V62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,39 +531,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xd699290087d2a48cd7892b469be90f5badfc464f7b0c8e88bcf43ad57fe9e0e5</t>
+          <t>0xe120c3d74babbe911760748d765692a0aedf1e1b17ace3e84541e902469ac97d</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x7FBBAf1D0066D0f087b3686cAfd17b3B4A25Aa4b</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>7.16863</t>
+          <t>1.04</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.345</t>
+          <t>1.5663</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>FC Nordsjælland -1.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -571,27 +563,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>FC Nordsjælland vs Randers FC</t>
+          <t>Odense BK vs Sonderjyske</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>FC Nordsjælland</t>
+          <t>Odense BK</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Randers FC</t>
+          <t>Sonderjyske</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x21cc7fc7dc172ea037bb4b7e06435d4eab87d2b9eb7d07444e82080b40de780f</t>
+          <t>0x8de61d36739ddb5bdf4a23c7744a220bcf5561255580d9cf5d474d0c20cddea6</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19592303</t>
+          <t>L19592309</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +608,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785634632</t>
+          <t>1785650300</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785672000</t>
+          <t>1785776400</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>20.778638</t>
+          <t>1.836645</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,39 +635,31 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x7bc0645f83f558bd49d72ab5929e48a360bec86f5c1c80a0b36499e179f6bc90</t>
+          <t>0x68739407304f74311377f2a626ce2a825df036235ace919bf5594583028dd663</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>9.08</t>
+          <t>5.99</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.1775</t>
+          <t>1.2525</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -683,27 +667,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Lyngby vs Aarhus AGF</t>
+          <t>FC Nordsjælland vs Randers FC</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Lyngby</t>
+          <t>FC Nordsjælland</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Aarhus AGF</t>
+          <t>Randers FC</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x2c1096977a572debdbc4134b01ca6c6adf49b6eaa39cf8725241774929205c38</t>
+          <t>0xee72621ab63112cc8034093022e9286514151b46f9608c676dccf64648d7a1e2</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19592306</t>
+          <t>L19592303</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -728,17 +712,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785605691</t>
+          <t>1785645887</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1785600000</t>
+          <t>1785672000</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>51.15493</t>
+          <t>23.722772</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,39 +739,31 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xa319add42d7daca25f7ce612631721cb63e4e5ba5f3632b1a9f0aaec034233b4</t>
+          <t>0xf9ffad34157551319e43915bc587ce619ee2058a6fc9bbac1ccc51fc6324685c</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>160.03209</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.1825</t>
+          <t>1.9075</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -795,27 +771,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Lyngby vs Aarhus AGF</t>
+          <t>FC Midtjylland vs AC Horsens</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Lyngby</t>
+          <t>FC Midtjylland</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Aarhus AGF</t>
+          <t>AC Horsens</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x2c1096977a572debdbc4134b01ca6c6adf49b6eaa39cf8725241774929205c38</t>
+          <t>0x06e37a2d11a20989c8d86887cfdf77d942e5715d3b7379239c05c651cb346c68</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19592306</t>
+          <t>L19592302</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -840,17 +816,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785605676</t>
+          <t>1785645227</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1785600000</t>
+          <t>1785672000</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>5.479452</t>
+          <t>176.343901</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,7 +843,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xa4126a9e4494025031a85230fa4ae999142b42db89a2b4bfa25dedb64fa10361</t>
+          <t>0xd699290087d2a48cd7892b469be90f5badfc464f7b0c8e88bcf43ad57fe9e0e5</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -875,23 +851,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>15.86</t>
+          <t>7.16863</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.37</t>
+          <t>1.345</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>FC Nordsjælland -1.5</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -899,27 +883,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Lyngby vs Aarhus AGF</t>
+          <t>FC Nordsjælland vs Randers FC</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Lyngby</t>
+          <t>FC Nordsjælland</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Aarhus AGF</t>
+          <t>Randers FC</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x2c79dee42344af7b9246e60dc88e4e41c38fed19c8d52ae01c0cfc28609e9d76</t>
+          <t>0x21cc7fc7dc172ea037bb4b7e06435d4eab87d2b9eb7d07444e82080b40de780f</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19592306</t>
+          <t>L19592303</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -944,17 +928,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785604733</t>
+          <t>1785634632</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1785600000</t>
+          <t>1785672000</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>42.864865</t>
+          <t>20.778638</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,23 +955,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xae3080012711fb7f128ce737fc1040d8f46c353403aac355fceefef37455ef29</t>
+          <t>0x7bc0645f83f558bd49d72ab5929e48a360bec86f5c1c80a0b36499e179f6bc90</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x9E844C0c1B06456051E307CC2d6F747387398Dda</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>67.42854</t>
+          <t>9.08</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.7925</t>
+          <t>1.1775</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -995,7 +983,11 @@
           <t>Under/Over (3.5)</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -1048,7 +1040,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785604244</t>
+          <t>1785605691</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1058,7 +1050,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>85.083331</t>
+          <t>51.15493</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,23 +1067,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x991c66883f3babf09f89f2ddc2edbe3e7fe5aca0b354a64851cdb157d9584476</t>
+          <t>0xa319add42d7daca25f7ce612631721cb63e4e5ba5f3632b1a9f0aaec034233b4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x9E844C0c1B06456051E307CC2d6F747387398Dda</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>18.87999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.7925</t>
+          <t>1.1825</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1099,7 +1095,11 @@
           <t>Under/Over (3.5)</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785604241</t>
+          <t>1785605676</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>23.823331</t>
+          <t>5.479452</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,7 +1179,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xbcce72b29126f648e0a9a41af52ca65b337ca9469b2fa8e14b40d240e70553cf</t>
+          <t>0xa4126a9e4494025031a85230fa4ae999142b42db89a2b4bfa25dedb64fa10361</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1187,31 +1187,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15.86</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.22</t>
+          <t>1.37</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -1234,7 +1226,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x2c1096977a572debdbc4134b01ca6c6adf49b6eaa39cf8725241774929205c38</t>
+          <t>0x2c79dee42344af7b9246e60dc88e4e41c38fed19c8d52ae01c0cfc28609e9d76</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1264,7 +1256,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785604232</t>
+          <t>1785604733</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1274,7 +1266,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>45.454545</t>
+          <t>42.864865</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1291,7 +1283,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xb1f7c6db5b79d433d261821aef5cde6942f2794c9653159c5a1e77c9021007f3</t>
+          <t>0xae3080012711fb7f128ce737fc1040d8f46c353403aac355fceefef37455ef29</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1302,12 +1294,12 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>67.42854</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.7812</t>
+          <t>1.7925</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1368,7 +1360,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785604165</t>
+          <t>1785604244</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1378,7 +1370,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>128.0</t>
+          <t>85.083331</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1395,7 +1387,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x70c28cd2394cb1cd4bfbe937655e46156c19918e5e8a6a73b3f54ed43f4780d4</t>
+          <t>0x991c66883f3babf09f89f2ddc2edbe3e7fe5aca0b354a64851cdb157d9584476</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1406,12 +1398,12 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>18.87999</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.7812</t>
+          <t>1.7925</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1472,7 +1464,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785604165</t>
+          <t>1785604241</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1482,7 +1474,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>128.0</t>
+          <t>23.823331</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1499,12 +1491,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x3b18d977a7fd211a0f9e5e278f1127cba12e28ff08b808655154498f731a7764</t>
+          <t>0xbcce72b29126f648e0a9a41af52ca65b337ca9469b2fa8e14b40d240e70553cf</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x9E844C0c1B06456051E307CC2d6F747387398Dda</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1514,47 +1506,47 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.625</t>
+          <t>1.22</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Superliga</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Lyngby vs Aarhus AGF</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Lyngby</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
           <t>Aarhus AGF</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Superliga</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Lyngby vs Aarhus AGF</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Lyngby</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Aarhus AGF</t>
-        </is>
-      </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
+          <t>0x2c1096977a572debdbc4134b01ca6c6adf49b6eaa39cf8725241774929205c38</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1584,7 +1576,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785603398</t>
+          <t>1785604232</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1594,7 +1586,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>160.0</t>
+          <t>45.454545</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1611,28 +1603,28 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x29a960a301fde84f871ab5479215a370ef7cd4221add949ccdbf6437d90bee66</t>
+          <t>0xb1f7c6db5b79d433d261821aef5cde6942f2794c9653159c5a1e77c9021007f3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x9E844C0c1B06456051E307CC2d6F747387398Dda</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.67</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.3875</t>
+          <t>1.7812</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1658,7 +1650,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
+          <t>0x2c1096977a572debdbc4134b01ca6c6adf49b6eaa39cf8725241774929205c38</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1688,7 +1680,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785603360</t>
+          <t>1785604165</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1698,7 +1690,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>4.309677</t>
+          <t>128.0</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1715,39 +1707,31 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x252690fda143cd5cffffe7acc9d80be88e7f1b017e8a4b8e7bb0c9a3e20dcc92</t>
+          <t>0x70c28cd2394cb1cd4bfbe937655e46156c19918e5e8a6a73b3f54ed43f4780d4</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x9E844C0c1B06456051E307CC2d6F747387398Dda</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>3.32</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.39</t>
+          <t>1.7812</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Lyngby +0.5</t>
-        </is>
-      </c>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -1770,7 +1754,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xebf51dcb3b623eff5755a2aaedf48104b7c37c1031827992daded7df498eb858</t>
+          <t>0x2c1096977a572debdbc4134b01ca6c6adf49b6eaa39cf8725241774929205c38</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1800,7 +1784,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785603312</t>
+          <t>1785604165</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1810,7 +1794,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>8.512821</t>
+          <t>128.0</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1827,23 +1811,27 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xce388e858e0ee1eeb493c07c312f91158610729f2d3d7ea07014063791a035f1</t>
+          <t>0x3b18d977a7fd211a0f9e5e278f1127cba12e28ff08b808655154498f731a7764</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
+          <t>0x9E844C0c1B06456051E307CC2d6F747387398Dda</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1.38998</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.8988</t>
+          <t>1.625</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1851,7 +1839,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Aarhus AGF</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -1859,27 +1851,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>FC Midtjylland vs AC Horsens</t>
+          <t>Lyngby vs Aarhus AGF</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>FC Midtjylland</t>
+          <t>Lyngby</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>AC Horsens</t>
+          <t>Aarhus AGF</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x06e37a2d11a20989c8d86887cfdf77d942e5715d3b7379239c05c651cb346c68</t>
+          <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19592302</t>
+          <t>L19592306</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1904,17 +1896,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785603282</t>
+          <t>1785603398</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1785672000</t>
+          <t>1785600000</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1.54657</t>
+          <t>160.0</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1931,7 +1923,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xa258d254c983ab7192759168951cc17ca08b00cdbd0f1848992fb45c3774dcdd</t>
+          <t>0x29a960a301fde84f871ab5479215a370ef7cd4221add949ccdbf6437d90bee66</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1942,17 +1934,17 @@
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>34.03</t>
+          <t>1.67</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.405</t>
+          <t>1.3875</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1978,7 +1970,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x49526fbc0f036a835cadb6ed200a2149c33841e9732da24e1a26ae104dbca7c3</t>
+          <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2008,7 +2000,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785602596</t>
+          <t>1785603360</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2018,7 +2010,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>84.024691</t>
+          <t>4.309677</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2035,7 +2027,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xe5932133cd6dd1a673902f8878c284852594ee9d0f3cea4416b672143b920008</t>
+          <t>0x252690fda143cd5cffffe7acc9d80be88e7f1b017e8a4b8e7bb0c9a3e20dcc92</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2050,39 +2042,39 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>14.2</t>
+          <t>3.32</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.1625</t>
+          <t>1.39</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (0.5)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
+          <t>Lyngby +0.5</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Superliga</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Lyngby vs Aarhus AGF</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
           <t>Lyngby</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Superliga</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Lyngby vs Aarhus AGF</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Lyngby</t>
-        </is>
-      </c>
       <c r="K16" t="inlineStr">
         <is>
           <t>Aarhus AGF</t>
@@ -2090,7 +2082,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xc70795d9541e318a1f58072592386f160a93a6c1e472c3a635af0c335cbe97fd</t>
+          <t>0xebf51dcb3b623eff5755a2aaedf48104b7c37c1031827992daded7df498eb858</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2120,7 +2112,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785602558</t>
+          <t>1785603312</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2130,7 +2122,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>87.384615</t>
+          <t>8.512821</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2147,7 +2139,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x6c47e3b5b9fe2a953f71ebc11060987f20d92b9f45088637990af9732f1e37d9</t>
+          <t>0xce388e858e0ee1eeb493c07c312f91158610729f2d3d7ea07014063791a035f1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2155,19 +2147,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>3.48</t>
+          <t>1.38998</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.1713</t>
+          <t>1.8988</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2175,11 +2163,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Lyngby</t>
-        </is>
-      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -2187,27 +2171,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Lyngby vs Aarhus AGF</t>
+          <t>FC Midtjylland vs AC Horsens</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Lyngby</t>
+          <t>FC Midtjylland</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Aarhus AGF</t>
+          <t>AC Horsens</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0xc70795d9541e318a1f58072592386f160a93a6c1e472c3a635af0c335cbe97fd</t>
+          <t>0x06e37a2d11a20989c8d86887cfdf77d942e5715d3b7379239c05c651cb346c68</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>L19592306</t>
+          <t>L19592302</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2232,17 +2216,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785602406</t>
+          <t>1785603282</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>1785600000</t>
+          <t>1785672000</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>20.321168</t>
+          <t>1.54657</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2259,7 +2243,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0xdf40cd66f398b60374d5f662a56dcca16ac17a6436e2af510172e4794b7a1b91</t>
+          <t>0xa258d254c983ab7192759168951cc17ca08b00cdbd0f1848992fb45c3774dcdd</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2267,46 +2251,38 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>34.03</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.1713</t>
+          <t>1.405</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Superliga</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Lyngby vs Aarhus AGF</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
         <is>
           <t>Lyngby</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Superliga</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Lyngby vs Aarhus AGF</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Lyngby</t>
-        </is>
-      </c>
       <c r="K18" t="inlineStr">
         <is>
           <t>Aarhus AGF</t>
@@ -2314,7 +2290,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xc70795d9541e318a1f58072592386f160a93a6c1e472c3a635af0c335cbe97fd</t>
+          <t>0x49526fbc0f036a835cadb6ed200a2149c33841e9732da24e1a26ae104dbca7c3</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2344,7 +2320,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785602395</t>
+          <t>1785602596</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2354,7 +2330,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>6.014599</t>
+          <t>84.024691</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2371,7 +2347,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x542c9ee3ba50079371d69b225a2c8db6ff22236586c78ca30be352ec364ea7b8</t>
+          <t>0xe5932133cd6dd1a673902f8878c284852594ee9d0f3cea4416b672143b920008</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2379,15 +2355,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>172.93998</t>
+          <t>14.2</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.7625</t>
+          <t>1.1625</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2395,7 +2375,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Lyngby</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -2448,7 +2432,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785602314</t>
+          <t>1785602558</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2458,7 +2442,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>226.806531</t>
+          <t>87.384615</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2475,7 +2459,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x32404e24a01d0f39a33dae82f210cebc058f485f67257ccb519209e9cbf31e9c</t>
+          <t>0x6c47e3b5b9fe2a953f71ebc11060987f20d92b9f45088637990af9732f1e37d9</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2483,23 +2467,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0.00164</t>
+          <t>3.48</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.3487</t>
+          <t>1.1713</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Lyngby</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -2522,7 +2514,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x49526fbc0f036a835cadb6ed200a2149c33841e9732da24e1a26ae104dbca7c3</t>
+          <t>0xc70795d9541e318a1f58072592386f160a93a6c1e472c3a635af0c335cbe97fd</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2552,7 +2544,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785602219</t>
+          <t>1785602406</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2562,7 +2554,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>0.004703</t>
+          <t>20.321168</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2579,12 +2571,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x290c4be361999ca74e5190289205640fbde3883451b1cda08ad62da22e8bd73b</t>
+          <t>0xdf40cd66f398b60374d5f662a56dcca16ac17a6436e2af510172e4794b7a1b91</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2594,12 +2586,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>624.35</t>
+          <t>1.03</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.3725</t>
+          <t>1.1713</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2664,7 +2656,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1785601653</t>
+          <t>1785602395</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2674,7 +2666,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1676.107383</t>
+          <t>6.014599</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2691,7 +2683,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x5517a0cb27f87b517d9c76752f21658282493c534149cc6677898069a4d005c9</t>
+          <t>0x542c9ee3ba50079371d69b225a2c8db6ff22236586c78ca30be352ec364ea7b8</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2702,17 +2694,17 @@
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>12.35</t>
+          <t>172.93998</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.2463</t>
+          <t>1.7625</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -2738,7 +2730,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0xc6f8347a20a2fe84c2a09e64811d07034a4a3c889bcb651f9a9cb419b2085a6b</t>
+          <t>0xc70795d9541e318a1f58072592386f160a93a6c1e472c3a635af0c335cbe97fd</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2768,7 +2760,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785600726</t>
+          <t>1785602314</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2778,7 +2770,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>50.152284</t>
+          <t>226.806531</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2795,39 +2787,31 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x4d460fa043df63c7e0e47a0d4fc5206aa6128a136bb6b2e36dcf6df4c37e5340</t>
+          <t>0x32404e24a01d0f39a33dae82f210cebc058f485f67257ccb519209e9cbf31e9c</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>61.2</t>
+          <t>0.00164</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.775</t>
+          <t>1.3487</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Asian Handicap (1)</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Lyngby +1</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -2850,7 +2834,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0xe699f8c24bc0df7c6904cb93a6259e9884ce88e8a6c08e345b0b23111f84a362</t>
+          <t>0x49526fbc0f036a835cadb6ed200a2149c33841e9732da24e1a26ae104dbca7c3</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2880,7 +2864,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785600074</t>
+          <t>1785602219</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2890,7 +2874,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>78.967742</t>
+          <t>0.004703</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2907,7 +2891,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x43032cc369d485f1c4840ed9e54e060c40aad483cde4aab6d9526f28e80c6d8c</t>
+          <t>0x290c4be361999ca74e5190289205640fbde3883451b1cda08ad62da22e8bd73b</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2915,15 +2899,19 @@
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>21.73999</t>
+          <t>624.35</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.6587</t>
+          <t>1.3725</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2931,7 +2919,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Lyngby</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -2984,7 +2976,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785599892</t>
+          <t>1785601653</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -2994,7 +2986,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>33.001882</t>
+          <t>1676.107383</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3011,39 +3003,31 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x477b1e59ff24b6874af79bd81ca84826e775addebb73c0455ce8f316764d24f1</t>
+          <t>0x5517a0cb27f87b517d9c76752f21658282493c534149cc6677898069a4d005c9</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10.02</t>
+          <t>12.35</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.4788</t>
+          <t>1.2463</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Superliga</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Lyngby 0</t>
-        </is>
-      </c>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -3066,7 +3050,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0xc6bfa4ca006143bd24c5bf127f777b5499a188178e3675286701690a0a4cb87c</t>
+          <t>0xc6f8347a20a2fe84c2a09e64811d07034a4a3c889bcb651f9a9cb419b2085a6b</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3096,7 +3080,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1785599755</t>
+          <t>1785600726</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3106,7 +3090,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>20.929504</t>
+          <t>50.152284</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3123,12 +3107,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x7357b0eab452a7acd8e946ea7273ae514c279e3347a90627d1a9585d3c5843c5</t>
+          <t>0x4d460fa043df63c7e0e47a0d4fc5206aa6128a136bb6b2e36dcf6df4c37e5340</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3138,22 +3122,22 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10.97942</t>
+          <t>61.2</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.3562</t>
+          <t>1.775</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Asian Handicap (1)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Lyngby +1</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3178,7 +3162,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x2c1096977a572debdbc4134b01ca6c6adf49b6eaa39cf8725241774929205c38</t>
+          <t>0xe699f8c24bc0df7c6904cb93a6259e9884ce88e8a6c08e345b0b23111f84a362</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3208,7 +3192,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1785599673</t>
+          <t>1785600074</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3218,7 +3202,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>30.819425</t>
+          <t>78.967742</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3235,7 +3219,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x2b7fd038168881dd534ca275f5ed230a57acd5fa3a0ebb3af697ff456cfaf7a6</t>
+          <t>0x43032cc369d485f1c4840ed9e54e060c40aad483cde4aab6d9526f28e80c6d8c</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3243,19 +3227,15 @@
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>17.39</t>
+          <t>21.73999</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.3475</t>
+          <t>1.6587</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3263,26 +3243,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Superliga</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Lyngby vs Aarhus AGF</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
         <is>
           <t>Lyngby</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Superliga</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>Lyngby vs Aarhus AGF</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>Lyngby</t>
-        </is>
-      </c>
       <c r="K27" t="inlineStr">
         <is>
           <t>Aarhus AGF</t>
@@ -3320,7 +3296,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1785599575</t>
+          <t>1785599892</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3330,7 +3306,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>50.043165</t>
+          <t>33.001882</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3347,12 +3323,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x601c8848886fb886b0180b4e4fbd1406da8b2dfd9ca0bbd4217323e85c7bbb54</t>
+          <t>0x477b1e59ff24b6874af79bd81ca84826e775addebb73c0455ce8f316764d24f1</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3362,22 +3338,22 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>24.27559</t>
+          <t>10.02</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.5837</t>
+          <t>1.4788</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Superliga</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Lyngby 0</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -3402,7 +3378,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0x49526fbc0f036a835cadb6ed200a2149c33841e9732da24e1a26ae104dbca7c3</t>
+          <t>0xc6bfa4ca006143bd24c5bf127f777b5499a188178e3675286701690a0a4cb87c</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3432,7 +3408,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1785598976</t>
+          <t>1785599755</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3442,7 +3418,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>41.585593</t>
+          <t>20.929504</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3459,7 +3435,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0xfbaa9c24b9510ae8e373ef34d1ecad4c6f03b0ecd50f5f1dabf8d96eac05045e</t>
+          <t>0x7357b0eab452a7acd8e946ea7273ae514c279e3347a90627d1a9585d3c5843c5</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3474,22 +3450,22 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>17.52</t>
+          <t>10.97942</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.4575</t>
+          <t>1.3562</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Over 3.0</t>
+          <t>Over 3.5</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -3514,7 +3490,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0xe11a19f75d36d5d6419b78d721044e6cb26bbb94b7ffe966a3db535ef797b2a0</t>
+          <t>0x2c1096977a572debdbc4134b01ca6c6adf49b6eaa39cf8725241774929205c38</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3544,7 +3520,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1785598938</t>
+          <t>1785599673</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3554,7 +3530,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>38.295082</t>
+          <t>30.819425</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3571,12 +3547,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0xac28d9e7fe7cec2c18df8cb76f74d655123de61c1db7f9b657ef28517696a744</t>
+          <t>0x2b7fd038168881dd534ca275f5ed230a57acd5fa3a0ebb3af697ff456cfaf7a6</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3586,22 +3562,22 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>3.31</t>
+          <t>17.39</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.5837</t>
+          <t>1.3475</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Lyngby</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3626,7 +3602,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0x49526fbc0f036a835cadb6ed200a2149c33841e9732da24e1a26ae104dbca7c3</t>
+          <t>0xc70795d9541e318a1f58072592386f160a93a6c1e472c3a635af0c335cbe97fd</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3656,7 +3632,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1785598938</t>
+          <t>1785599575</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3666,7 +3642,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>5.670236</t>
+          <t>50.043165</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3683,7 +3659,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x145f1890db61a13e6074edd94e8c7d3505a6648ce87181ddb463661f63e4ac71</t>
+          <t>0x601c8848886fb886b0180b4e4fbd1406da8b2dfd9ca0bbd4217323e85c7bbb54</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3698,22 +3674,22 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>7.24</t>
+          <t>24.27559</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.355</t>
+          <t>1.5837</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3738,7 +3714,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0x2c1096977a572debdbc4134b01ca6c6adf49b6eaa39cf8725241774929205c38</t>
+          <t>0x49526fbc0f036a835cadb6ed200a2149c33841e9732da24e1a26ae104dbca7c3</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -3768,7 +3744,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1785598938</t>
+          <t>1785598976</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3778,7 +3754,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>20.394366</t>
+          <t>41.585593</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3795,7 +3771,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x83a64669b6d24f6b2bfa8fb7f99efe76976776e0c4bc16d9353af65cab35d8ea</t>
+          <t>0xfbaa9c24b9510ae8e373ef34d1ecad4c6f03b0ecd50f5f1dabf8d96eac05045e</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3810,22 +3786,22 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>66.45</t>
+          <t>17.52</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.475</t>
+          <t>1.4575</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Superliga</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Lyngby 0</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3850,7 +3826,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0xc6bfa4ca006143bd24c5bf127f777b5499a188178e3675286701690a0a4cb87c</t>
+          <t>0xe11a19f75d36d5d6419b78d721044e6cb26bbb94b7ffe966a3db535ef797b2a0</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3880,7 +3856,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1785598157</t>
+          <t>1785598938</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3890,7 +3866,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>139.894737</t>
+          <t>38.295082</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3907,7 +3883,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0xfa4501eddd39f3bc6b2b0b6e89ccf2a76e8e3a21c4ca206725c5debad85d7f16</t>
+          <t>0xac28d9e7fe7cec2c18df8cb76f74d655123de61c1db7f9b657ef28517696a744</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3915,23 +3891,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>1.86</t>
+          <t>3.31</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.6212</t>
+          <t>1.5837</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -3954,7 +3938,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
+          <t>0x49526fbc0f036a835cadb6ed200a2149c33841e9732da24e1a26ae104dbca7c3</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -3984,7 +3968,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1785597943</t>
+          <t>1785598938</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -3994,7 +3978,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>2.993964</t>
+          <t>5.670236</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4011,7 +3995,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x1fef8c656712a6c033b201778e6ea23411792a11a8364435015c2501f5bcf6b7</t>
+          <t>0x145f1890db61a13e6074edd94e8c7d3505a6648ce87181ddb463661f63e4ac71</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4019,23 +4003,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>71.62</t>
+          <t>7.24</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.6187</t>
+          <t>1.355</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr"/>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -4058,7 +4050,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
+          <t>0x2c1096977a572debdbc4134b01ca6c6adf49b6eaa39cf8725241774929205c38</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -4088,7 +4080,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785595979</t>
+          <t>1785598938</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4098,7 +4090,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>115.749495</t>
+          <t>20.394366</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4115,23 +4107,27 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x8d26b053739a961371fc982398bb23a61268a2a763247c7dcab222a06e9f01ab</t>
+          <t>0x83a64669b6d24f6b2bfa8fb7f99efe76976776e0c4bc16d9353af65cab35d8ea</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>66.45</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.5288</t>
+          <t>1.475</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4139,7 +4135,11 @@
           <t>Superliga</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Lyngby 0</t>
+        </is>
+      </c>
       <c r="H35" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -4162,7 +4162,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0x1baa4864a899a4f985ce46660f0cf1b4b06170bd254c29ad505c1041d2d5d9b9</t>
+          <t>0xc6bfa4ca006143bd24c5bf127f777b5499a188178e3675286701690a0a4cb87c</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -4192,7 +4192,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1785595943</t>
+          <t>1785598157</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>9.456265</t>
+          <t>139.894737</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4219,28 +4219,28 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x8b0e287b826a0a08876c7fc45b8edd6e8b1860b00baa9b8188437cf82c03712c</t>
+          <t>0xfa4501eddd39f3bc6b2b0b6e89ccf2a76e8e3a21c4ca206725c5debad85d7f16</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1.86</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.5288</t>
+          <t>1.6212</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Superliga</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
@@ -4266,7 +4266,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0xc6bfa4ca006143bd24c5bf127f777b5499a188178e3675286701690a0a4cb87c</t>
+          <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4296,7 +4296,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1785595941</t>
+          <t>1785597943</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4306,7 +4306,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>9.456265</t>
+          <t>2.993964</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4323,28 +4323,28 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0xdfd6bb1e051c4e6625f5e08f938d63a5fdc9545c9700a3d0b437d6135415c8ff</t>
+          <t>0x1fef8c656712a6c033b201778e6ea23411792a11a8364435015c2501f5bcf6b7</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>71.62</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.5288</t>
+          <t>1.6187</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Superliga</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
@@ -4370,7 +4370,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0x1baa4864a899a4f985ce46660f0cf1b4b06170bd254c29ad505c1041d2d5d9b9</t>
+          <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4400,7 +4400,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1785595939</t>
+          <t>1785595979</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4410,7 +4410,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>9.456265</t>
+          <t>115.749495</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4427,18 +4427,18 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0xc2cac2e0309c6b93054ecfb0370f7eac3dd858f41b476e1389d2973c80f4e426</t>
+          <t>0x8d26b053739a961371fc982398bb23a61268a2a763247c7dcab222a06e9f01ab</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>15.84286</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -4474,7 +4474,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0xc6bfa4ca006143bd24c5bf127f777b5499a188178e3675286701690a0a4cb87c</t>
+          <t>0x1baa4864a899a4f985ce46660f0cf1b4b06170bd254c29ad505c1041d2d5d9b9</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4504,7 +4504,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1785595933</t>
+          <t>1785595943</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>29.962856</t>
+          <t>9.456265</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4531,18 +4531,18 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x8d090f4e722db24c40e4e198e16c314766056fc6f3bb6961d1ba589139c11932</t>
+          <t>0x8b0e287b826a0a08876c7fc45b8edd6e8b1860b00baa9b8188437cf82c03712c</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>15.84286</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -4578,7 +4578,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0x1baa4864a899a4f985ce46660f0cf1b4b06170bd254c29ad505c1041d2d5d9b9</t>
+          <t>0xc6bfa4ca006143bd24c5bf127f777b5499a188178e3675286701690a0a4cb87c</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4608,7 +4608,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1785595933</t>
+          <t>1785595941</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>29.962856</t>
+          <t>9.456265</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4635,18 +4635,18 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x973562122e8c9af30ad3b521dcdab6041ac8a1a4ab5e3ba032a608be6cc060ee</t>
+          <t>0xdfd6bb1e051c4e6625f5e08f938d63a5fdc9545c9700a3d0b437d6135415c8ff</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>14.11495</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -4682,7 +4682,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0xc6bfa4ca006143bd24c5bf127f777b5499a188178e3675286701690a0a4cb87c</t>
+          <t>0x1baa4864a899a4f985ce46660f0cf1b4b06170bd254c29ad505c1041d2d5d9b9</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -4712,7 +4712,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1785595932</t>
+          <t>1785595939</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4722,7 +4722,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>26.694941</t>
+          <t>9.456265</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4739,7 +4739,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0x10e039f9beee231795695cfaea431df60f459f016cbdab1dde259671236b3a0b</t>
+          <t>0xc2cac2e0309c6b93054ecfb0370f7eac3dd858f41b476e1389d2973c80f4e426</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4750,7 +4750,7 @@
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>14.11495</t>
+          <t>15.84286</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -4786,7 +4786,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0x1baa4864a899a4f985ce46660f0cf1b4b06170bd254c29ad505c1041d2d5d9b9</t>
+          <t>0xc6bfa4ca006143bd24c5bf127f777b5499a188178e3675286701690a0a4cb87c</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1785595931</t>
+          <t>1785595933</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4826,7 +4826,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>26.694941</t>
+          <t>29.962856</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4843,28 +4843,28 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0x45db1f79a8782bebdfa9ca6aa320b1a17d3135226a89444f15497cbff330db86</t>
+          <t>0x8d090f4e722db24c40e4e198e16c314766056fc6f3bb6961d1ba589139c11932</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>95.03</t>
+          <t>15.84286</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.6138</t>
+          <t>1.5288</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Superliga</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
@@ -4890,7 +4890,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
+          <t>0x1baa4864a899a4f985ce46660f0cf1b4b06170bd254c29ad505c1041d2d5d9b9</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -4920,7 +4920,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1785595862</t>
+          <t>1785595933</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -4930,7 +4930,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>154.835031</t>
+          <t>29.962856</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -4947,7 +4947,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0xf3fdbdc2cac9ca0f1daa7415d14604691092e7800dd73326a0964c8f59ca2138</t>
+          <t>0x973562122e8c9af30ad3b521dcdab6041ac8a1a4ab5e3ba032a608be6cc060ee</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4955,19 +4955,15 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>22.59</t>
+          <t>14.11495</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.465</t>
+          <t>1.5288</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -4975,11 +4971,7 @@
           <t>Superliga</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Lyngby 0</t>
-        </is>
-      </c>
+      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -5032,7 +5024,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1785595860</t>
+          <t>1785595932</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -5042,7 +5034,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>48.580645</t>
+          <t>26.694941</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5059,7 +5051,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0x0967cd6c0d9af8144107705eeb20dd2d7194c5d7b4b7c027264e753b60b9c154</t>
+          <t>0x10e039f9beee231795695cfaea431df60f459f016cbdab1dde259671236b3a0b</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -5067,19 +5059,15 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>22.51</t>
+          <t>14.11495</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.4638</t>
+          <t>1.5288</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -5087,26 +5075,22 @@
           <t>Superliga</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Superliga</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Lyngby vs Aarhus AGF</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
         <is>
           <t>Lyngby</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Superliga</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>Lyngby vs Aarhus AGF</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>Lyngby</t>
-        </is>
-      </c>
       <c r="K44" t="inlineStr">
         <is>
           <t>Aarhus AGF</t>
@@ -5144,7 +5128,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1785595859</t>
+          <t>1785595931</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -5154,7 +5138,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>48.539084</t>
+          <t>26.694941</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5171,27 +5155,23 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0x706b1c37ec80342daeeb16bff6cc06fbccfd683f08a0b3abf5ca007450e34f9c</t>
+          <t>0x45db1f79a8782bebdfa9ca6aa320b1a17d3135226a89444f15497cbff330db86</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>42.34254</t>
+          <t>95.03</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t>1.6138</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -5199,26 +5179,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Superliga</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Lyngby vs Aarhus AGF</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
         <is>
           <t>Lyngby</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Superliga</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>Lyngby vs Aarhus AGF</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>Lyngby</t>
-        </is>
-      </c>
       <c r="K45" t="inlineStr">
         <is>
           <t>Aarhus AGF</t>
@@ -5226,7 +5202,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>0xc70795d9541e318a1f58072592386f160a93a6c1e472c3a635af0c335cbe97fd</t>
+          <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -5256,7 +5232,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1785595852</t>
+          <t>1785595862</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
@@ -5266,7 +5242,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>124.536882</t>
+          <t>154.835031</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5283,7 +5259,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0x21acd3ca11d62dc03aebf7b22c220b68d622c3d52554514f2f52b6a3e5bc9f60</t>
+          <t>0xf3fdbdc2cac9ca0f1daa7415d14604691092e7800dd73326a0964c8f59ca2138</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -5298,12 +5274,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>654.51</t>
+          <t>22.59</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>1.4612</t>
+          <t>1.465</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -5368,7 +5344,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>1785595851</t>
+          <t>1785595860</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
@@ -5378,7 +5354,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>1418.99187</t>
+          <t>48.580645</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -5395,31 +5371,39 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0x8b434998185c6a9addd0fe1e0c178bf530ba5701b2034a87f6c857c16d441516</t>
+          <t>0x0967cd6c0d9af8144107705eeb20dd2d7194c5d7b4b7c027264e753b60b9c154</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>149.49728</t>
+          <t>22.51</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>1.6162</t>
+          <t>1.4638</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr"/>
+          <t>Superliga</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Lyngby</t>
+        </is>
+      </c>
       <c r="H47" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -5427,27 +5411,27 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>FC Midtjylland vs AC Horsens</t>
+          <t>Lyngby vs Aarhus AGF</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>FC Midtjylland</t>
+          <t>Lyngby</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>AC Horsens</t>
+          <t>Aarhus AGF</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>0xa013f739a827929cea4ca4e900d54898cb7634201ed3ae3393a770ccd4cd7bb8</t>
+          <t>0x1baa4864a899a4f985ce46660f0cf1b4b06170bd254c29ad505c1041d2d5d9b9</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>L19592302</t>
+          <t>L19592306</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -5472,17 +5456,17 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>1785595320</t>
+          <t>1785595859</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>1785672000</t>
+          <t>1785600000</t>
         </is>
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>242.591935</t>
+          <t>48.539084</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -5499,23 +5483,27 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0xab8792791675520bdb29586e60eb75299824ebe7b0964794c7be9856885975de</t>
+          <t>0x706b1c37ec80342daeeb16bff6cc06fbccfd683f08a0b3abf5ca007450e34f9c</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>0x782Cc6beCa1D0C0AB2A174D52D450Da71d58DE73</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr"/>
+          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>42.34254</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>1.675</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5523,7 +5511,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Lyngby</t>
+        </is>
+      </c>
       <c r="H48" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -5576,7 +5568,7 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>1785580396</t>
+          <t>1785595852</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
@@ -5586,7 +5578,7 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>74.074074</t>
+          <t>124.536882</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -5603,31 +5595,39 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0x1ab5b66cefade53cf596ea6bd9159327ca7c4e2027b8de0475e55d660c08d8dc</t>
+          <t>0x21acd3ca11d62dc03aebf7b22c220b68d622c3d52554514f2f52b6a3e5bc9f60</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>3.01999</t>
+          <t>654.51</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>1.5837</t>
+          <t>1.4612</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr"/>
+          <t>Superliga</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Lyngby 0</t>
+        </is>
+      </c>
       <c r="H49" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -5650,7 +5650,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
+          <t>0xc6bfa4ca006143bd24c5bf127f777b5499a188178e3675286701690a0a4cb87c</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -5680,7 +5680,7 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>1785563440</t>
+          <t>1785595851</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
@@ -5690,7 +5690,7 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>5.17343</t>
+          <t>1418.99187</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -5707,28 +5707,28 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>0x4cbbec8ecea58f8d04cceef531c975f092958f08b2bd55f5ac8de753823859a3</t>
+          <t>0x8b434998185c6a9addd0fe1e0c178bf530ba5701b2034a87f6c857c16d441516</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
-          <t>3.47</t>
+          <t>149.49728</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>1.5813</t>
+          <t>1.6162</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G50" t="inlineStr"/>
@@ -5739,27 +5739,27 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Lyngby vs Aarhus AGF</t>
+          <t>FC Midtjylland vs AC Horsens</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Lyngby</t>
+          <t>FC Midtjylland</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Aarhus AGF</t>
+          <t>AC Horsens</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
+          <t>0xa013f739a827929cea4ca4e900d54898cb7634201ed3ae3393a770ccd4cd7bb8</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>L19592306</t>
+          <t>L19592302</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -5784,17 +5784,17 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>1785562648</t>
+          <t>1785595320</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>1785600000</t>
+          <t>1785672000</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>5.969892</t>
+          <t>242.591935</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -5811,23 +5811,23 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0x67e7bf060a191b56fd16241ed5a5679895fd02c3f6992310ce1faf945bc215b6</t>
+          <t>0xab8792791675520bdb29586e60eb75299824ebe7b0964794c7be9856885975de</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>0x237ee0a4bcC2D25604635C46468C61cfD7F51565</t>
+          <t>0x782Cc6beCa1D0C0AB2A174D52D450Da71d58DE73</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2.14</t>
+          <t>50</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>1.58</t>
+          <t>1.675</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5858,7 +5858,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
+          <t>0xc70795d9541e318a1f58072592386f160a93a6c1e472c3a635af0c335cbe97fd</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -5888,7 +5888,7 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>1785560493</t>
+          <t>1785580396</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
@@ -5898,7 +5898,7 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>3.689655</t>
+          <t>74.074074</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -5915,27 +5915,23 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>0xab1af8e8c30fab10a28210e3e6b783062097a4fef5cfb2ea83de4750c5373ddb</t>
+          <t>0x1ab5b66cefade53cf596ea6bd9159327ca7c4e2027b8de0475e55d660c08d8dc</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>0x90555F35378305Ad562A29916D311a0e1C741A32</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3.01999</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>1.435</t>
+          <t>1.5837</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -5943,31 +5939,27 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Superliga</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Lyngby vs Aarhus AGF</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Lyngby</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
         <is>
           <t>Aarhus AGF</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>Superliga</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>Lyngby vs Aarhus AGF</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>Lyngby</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>Aarhus AGF</t>
-        </is>
-      </c>
       <c r="L52" t="inlineStr">
         <is>
           <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
@@ -6000,7 +5992,7 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>1785560490</t>
+          <t>1785563440</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
@@ -6010,7 +6002,7 @@
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>22.988506</t>
+          <t>5.17343</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -6027,7 +6019,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>0xfd8acecfb0e46e008d1593a715bc4694742f1a72b4a0f5346c2ae1e09867cfe6</t>
+          <t>0x4cbbec8ecea58f8d04cceef531c975f092958f08b2bd55f5ac8de753823859a3</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -6035,19 +6027,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>17.55</t>
+          <t>3.47</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>1.3025</t>
+          <t>1.5813</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6055,26 +6043,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Superliga</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Lyngby vs Aarhus AGF</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
         <is>
           <t>Lyngby</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>Superliga</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>Lyngby vs Aarhus AGF</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>Lyngby</t>
-        </is>
-      </c>
       <c r="K53" t="inlineStr">
         <is>
           <t>Aarhus AGF</t>
@@ -6082,7 +6066,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>0xc70795d9541e318a1f58072592386f160a93a6c1e472c3a635af0c335cbe97fd</t>
+          <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -6112,7 +6096,7 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>1785560344</t>
+          <t>1785562648</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
@@ -6122,7 +6106,7 @@
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>58.016529</t>
+          <t>5.969892</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -6139,27 +6123,23 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>0x90f534a9fff131b27315577165c9e0e220d69a9b3b8482cf80327b3a63d197ba</t>
+          <t>0x67e7bf060a191b56fd16241ed5a5679895fd02c3f6992310ce1faf945bc215b6</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x237ee0a4bcC2D25604635C46468C61cfD7F51565</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
-          <t>0.0004</t>
+          <t>2.14</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>1.3025</t>
+          <t>1.58</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6167,26 +6147,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Superliga</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Lyngby vs Aarhus AGF</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
         <is>
           <t>Lyngby</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>Superliga</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>Lyngby vs Aarhus AGF</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>Lyngby</t>
-        </is>
-      </c>
       <c r="K54" t="inlineStr">
         <is>
           <t>Aarhus AGF</t>
@@ -6194,7 +6170,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>0xc70795d9541e318a1f58072592386f160a93a6c1e472c3a635af0c335cbe97fd</t>
+          <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -6224,7 +6200,7 @@
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>1785560343</t>
+          <t>1785560493</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
@@ -6234,7 +6210,7 @@
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>0.001322</t>
+          <t>3.689655</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -6251,23 +6227,27 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>0xbc6ea757f52e963de84e5dd1bb0a3a9a0ffc1e2774133abff95b9c4f2766dfce</t>
+          <t>0xab1af8e8c30fab10a28210e3e6b783062097a4fef5cfb2ea83de4750c5373ddb</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr"/>
+          <t>0x90555F35378305Ad562A29916D311a0e1C741A32</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>79.73</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>1.5713</t>
+          <t>1.435</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6275,7 +6255,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Aarhus AGF</t>
+        </is>
+      </c>
       <c r="H55" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -6328,7 +6312,7 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>1785560332</t>
+          <t>1785560490</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
@@ -6338,7 +6322,7 @@
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>139.571116</t>
+          <t>22.988506</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -6355,12 +6339,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>0xc2091d6709d3267143b7551e9bf0f634ad59da46580b096ae7180e9603ec2592</t>
+          <t>0xfd8acecfb0e46e008d1593a715bc4694742f1a72b4a0f5346c2ae1e09867cfe6</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -6370,12 +6354,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>17.55</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>1.2963</t>
+          <t>1.3025</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -6440,7 +6424,7 @@
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>1785551051</t>
+          <t>1785560344</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
@@ -6450,7 +6434,7 @@
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>121.518987</t>
+          <t>58.016529</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
@@ -6467,12 +6451,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>0xb7fcbce52de29f7db6fb4f41ad0da43f08c3dec3e184d58a2882cacd6dfaecfd</t>
+          <t>0x90f534a9fff131b27315577165c9e0e220d69a9b3b8482cf80327b3a63d197ba</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -6482,12 +6466,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.0004</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>1.4537</t>
+          <t>1.3025</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -6497,32 +6481,32 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
+          <t>Lyngby</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Superliga</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Lyngby vs Aarhus AGF</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Lyngby</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
           <t>Aarhus AGF</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>Superliga</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>Lyngby vs Aarhus AGF</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>Lyngby</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>Aarhus AGF</t>
-        </is>
-      </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
+          <t>0xc70795d9541e318a1f58072592386f160a93a6c1e472c3a635af0c335cbe97fd</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
@@ -6552,7 +6536,7 @@
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>1785513514</t>
+          <t>1785560343</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
@@ -6562,7 +6546,7 @@
       </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>2.203857</t>
+          <t>0.001322</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
@@ -6579,27 +6563,23 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>0x6e2898f2508a18394a27d0fccbbe6dcfbcfda464f076eafa6ee850e284c85b50</t>
+          <t>0xbc6ea757f52e963de84e5dd1bb0a3a9a0ffc1e2774133abff95b9c4f2766dfce</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2.22</t>
+          <t>79.73</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.5713</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -6607,11 +6587,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
           <t>Superliga</t>
@@ -6634,7 +6610,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>0x3b739c67fc6b69fa102f54ca6ebcb8b303dde9e5c25835c9afe89a9b97267e5e</t>
+          <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
@@ -6664,7 +6640,7 @@
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>1785346857</t>
+          <t>1785560332</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
@@ -6674,7 +6650,7 @@
       </c>
       <c r="T58" t="inlineStr">
         <is>
-          <t>7.4</t>
+          <t>139.571116</t>
         </is>
       </c>
       <c r="U58" t="inlineStr">
@@ -6691,110 +6667,446 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>0xc2091d6709d3267143b7551e9bf0f634ad59da46580b096ae7180e9603ec2592</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>0xc1BEa02928E7Dbb4b88c093f3EFC8FEcdC54334f</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>1.2963</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Lyngby</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Superliga</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Lyngby vs Aarhus AGF</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Lyngby</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Aarhus AGF</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>0xc70795d9541e318a1f58072592386f160a93a6c1e472c3a635af0c335cbe97fd</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>L19592306</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>1785551051</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>1785600000</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>121.518987</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>0xb7fcbce52de29f7db6fb4f41ad0da43f08c3dec3e184d58a2882cacd6dfaecfd</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>1.4537</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Aarhus AGF</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Superliga</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Lyngby vs Aarhus AGF</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Lyngby</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Aarhus AGF</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>L19592306</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>1785513514</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>1785600000</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>2.203857</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>0x6e2898f2508a18394a27d0fccbbe6dcfbcfda464f076eafa6ee850e284c85b50</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>2.22</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Superliga</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Lyngby vs Aarhus AGF</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Lyngby</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Aarhus AGF</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>0x3b739c67fc6b69fa102f54ca6ebcb8b303dde9e5c25835c9afe89a9b97267e5e</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>L19592306</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>1785346857</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>1785600000</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>0x864ae933266ffde8707769c32f9251b03c7600dc6768e603edb700f7d3f5d7cb</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B62" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="E62" t="inlineStr">
         <is>
           <t>1.555</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
+      <c r="F62" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr">
+      <c r="G62" t="inlineStr">
         <is>
           <t>Aarhus AGF</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>Superliga</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Superliga</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
         <is>
           <t>Lyngby vs Aarhus AGF</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr">
+      <c r="J62" t="inlineStr">
         <is>
           <t>Lyngby</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr">
+      <c r="K62" t="inlineStr">
         <is>
           <t>Aarhus AGF</t>
         </is>
       </c>
-      <c r="L59" t="inlineStr">
+      <c r="L62" t="inlineStr">
         <is>
           <t>0xf000d5daa6ad24f6820f826afb6b2a0e0aa80e629e469cc4bcdadb77cba654a5</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr">
+      <c r="M62" t="inlineStr">
         <is>
           <t>L19592306</t>
         </is>
       </c>
-      <c r="N59" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O59" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P59" t="inlineStr">
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q59" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R59" t="inlineStr">
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
         <is>
           <t>1785344233</t>
         </is>
       </c>
-      <c r="S59" t="inlineStr">
+      <c r="S62" t="inlineStr">
         <is>
           <t>1785600000</t>
         </is>
       </c>
-      <c r="T59" t="inlineStr">
+      <c r="T62" t="inlineStr">
         <is>
           <t>3.603604</t>
         </is>
       </c>
-      <c r="U59" t="inlineStr">
+      <c r="U62" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V59" t="inlineStr">
+      <c r="V62" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>